<commit_message>
feat: add matin, ghavabesh, ghavabesh-tafyiz, and ERA excel files
</commit_message>
<xml_diff>
--- a/ERA.xlsx
+++ b/ERA.xlsx
@@ -1,22 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matin\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="45" windowWidth="27795" windowHeight="12600"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$28</definedName>
+  </definedNames>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="113">
   <si>
     <t>تدارکات</t>
   </si>
@@ -60,27 +66,12 @@
     <t>مجوز خروج کالا</t>
   </si>
   <si>
-    <t>یک فیلد جدید اضافه شد به اسم مبدا خروج کالا تا فرایند هر فاز مربوط به مدیر فاز باشد</t>
-  </si>
-  <si>
-    <t>پیش فاکتور ضایعات</t>
-  </si>
-  <si>
     <t>فروش</t>
   </si>
   <si>
-    <t>یک سمت جدید اضاف شد ، سرپرست فروش ضایعات و از بقیه کارشناس ها جدا شد</t>
-  </si>
-  <si>
-    <t>اصلاح فرم درخواست ماشین آلات</t>
-  </si>
-  <si>
     <t>ترابری</t>
   </si>
   <si>
-    <t>راننده از لیست انتخاب شود ، زمان واقعی شروع و پایان کار اضاف شود</t>
-  </si>
-  <si>
     <t>حراست</t>
   </si>
   <si>
@@ -99,13 +90,283 @@
     <t>مجوز بارگیری</t>
   </si>
   <si>
-    <t>در فرم مجوزبارگیری امکان ثبت موسسه حمل اضافه شود</t>
+    <t>جدید</t>
+  </si>
+  <si>
+    <t>1405/03/30</t>
+  </si>
+  <si>
+    <t>1405/03/31</t>
+  </si>
+  <si>
+    <t>ایجاد و اصلاح فرآیند دلیل خروج اضطراری در مجوز خروج کالا</t>
+  </si>
+  <si>
+    <t>1405/02/24</t>
+  </si>
+  <si>
+    <t>تولید</t>
+  </si>
+  <si>
+    <t>درخواست خرید</t>
+  </si>
+  <si>
+    <t>اصلاح فرآیند درخواست خرید بر اساس نوع درخواست خرید</t>
+  </si>
+  <si>
+    <t>پیش فاکتور تا حواله فروش</t>
+  </si>
+  <si>
+    <t>اصلاح فرآیند فروش به تفکیک مرکز فروش</t>
+  </si>
+  <si>
+    <t>اصلاح تگ های پیش فاکتور برای واحد فروش به تفکیک مرکز فروش</t>
+  </si>
+  <si>
+    <t>اصلاح فرآیند مجوز خروج کالا بر اساس محل خروج (اضافه شدن مبدا خروج کالا)</t>
+  </si>
+  <si>
+    <t>اعلامیه پرداخت</t>
+  </si>
+  <si>
+    <t>حسابداری</t>
+  </si>
+  <si>
+    <t>اتوماتیک سازی صدور اعلامیه پرداخت برای تنه درخت ها</t>
+  </si>
+  <si>
+    <t>گزارش واریزی های دلاری</t>
+  </si>
+  <si>
+    <t>مطالبات</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اصلاح گزارش واریزی های دلاری </t>
+  </si>
+  <si>
+    <t>1405/02/26</t>
+  </si>
+  <si>
+    <t>فرمت های چاپی پیش فاکتور</t>
+  </si>
+  <si>
+    <t>1405/02/27</t>
+  </si>
+  <si>
+    <t>اصلاح فرمت های چاپی پیش فاکتور</t>
+  </si>
+  <si>
+    <t>کاوشگر محاسبه تولید</t>
+  </si>
+  <si>
+    <t>1405/02/28</t>
+  </si>
+  <si>
+    <t>اصلاح گزارش (کاوشگر) محاسبه تولید</t>
+  </si>
+  <si>
+    <t>1405/03/02</t>
+  </si>
+  <si>
+    <t>اصلاح گزارش</t>
+  </si>
+  <si>
+    <t>اصلاح گزارش خانم نجاران</t>
+  </si>
+  <si>
+    <t>1405/03/03</t>
+  </si>
+  <si>
+    <t>درخواست پاداش جریمه</t>
+  </si>
+  <si>
+    <t>اضافه نمودن نوع جدید (جریمه غیبت) به فرم پاداش/جریمه</t>
+  </si>
+  <si>
+    <t>گزارش فروش ماهیانه</t>
+  </si>
+  <si>
+    <t>1405/03/04</t>
+  </si>
+  <si>
+    <t>گردش کار مرخصی</t>
+  </si>
+  <si>
+    <t>اصلاح ساختار و گردش کار مرخصی برای واحد فروش</t>
+  </si>
+  <si>
+    <t>اصلاح گزارش آمار فروش ماهیانه خانم خزینه پور</t>
+  </si>
+  <si>
+    <t>1405/03/12</t>
+  </si>
+  <si>
+    <t>اصلاح گردش کار پیش فاکتور ضایعات</t>
+  </si>
+  <si>
+    <t>1405/03/20</t>
+  </si>
+  <si>
+    <t>کاوشگر اعلان</t>
+  </si>
+  <si>
+    <t>تعمیر و نگهداری</t>
+  </si>
+  <si>
+    <t>1405/03/23</t>
+  </si>
+  <si>
+    <t>ساخت گزارش (کاوشگر) اعلان برای آقای حسینی</t>
+  </si>
+  <si>
+    <t>گردش کار</t>
+  </si>
+  <si>
+    <t>ترخیص</t>
+  </si>
+  <si>
+    <t>1405/03/25</t>
+  </si>
+  <si>
+    <t>اصلاح ساختار گردش کار واحد ترخیص</t>
+  </si>
+  <si>
+    <t>اصلاح گزارش (کاوشگر) اعلان برای آقای حسینی</t>
+  </si>
+  <si>
+    <t>1405/03/24</t>
+  </si>
+  <si>
+    <t>گزارش مانده حساب مشتری</t>
+  </si>
+  <si>
+    <t>ساخت گزارش مانده حساب مشتری (بستانکاران) برای خانم نجاران جهت واحد فروش</t>
+  </si>
+  <si>
+    <t>اصلاح ویرایش موسسه حمل 2 جهت ثبت در مجوز بارگیری (وضعیت ثبت شده)</t>
+  </si>
+  <si>
+    <t>1405/04/01</t>
+  </si>
+  <si>
+    <t>اضافه کردن متن جدید شناسه دار شدن حساب ها</t>
+  </si>
+  <si>
+    <t>کارگزینی</t>
+  </si>
+  <si>
+    <t>اصلاح مشکل محاسبه گروهی فرم پاداش مصوب مدیریت</t>
+  </si>
+  <si>
+    <t>اضافه نمودن تاریخ و ساعت شروع و پایان شروع کار و خاتمه کار و انتخاب راننده از لیست</t>
+  </si>
+  <si>
+    <t>اصلاح دسترسی ویرایش ماموریت در حالت ثبت شده</t>
+  </si>
+  <si>
+    <t>اصلاح گزارش مانده حساب مشتری (بستانکاران) برای خانم نجاران جهت واحد فروش</t>
+  </si>
+  <si>
+    <t>پاداش تولید</t>
+  </si>
+  <si>
+    <t>اضافه نمودن نوع پاداش جدید به فرم پاداش تولید(پاداش تولید آتنا مارکت)</t>
+  </si>
+  <si>
+    <t>درخواست مرخصی</t>
+  </si>
+  <si>
+    <t>عمران</t>
+  </si>
+  <si>
+    <t>1405/04/07</t>
+  </si>
+  <si>
+    <t>اصلاح گردش درخواست کالا و مرخصی برای واحد عمران</t>
+  </si>
+  <si>
+    <t>اصلاح کالا</t>
+  </si>
+  <si>
+    <t>1405/04/11</t>
+  </si>
+  <si>
+    <t>مشکل تایید گروهی در فرم اصلاح کالا</t>
+  </si>
+  <si>
+    <t>درخواست ماموریت</t>
+  </si>
+  <si>
+    <t>اصلاح ساختار گردش کار مرخصی و ماموریت بر اساس ساختار مرخصی/ماموریت</t>
+  </si>
+  <si>
+    <t>1405/01/17</t>
+  </si>
+  <si>
+    <t>سرویس کارکنان</t>
+  </si>
+  <si>
+    <t>ساخت فرم سرویس کارکنان و تغییرات روزانه و گزارش تغییرات</t>
+  </si>
+  <si>
+    <t>دسترسی</t>
+  </si>
+  <si>
+    <t>اصلاح دسترسی های واحد حسابداری بر اساس گروه</t>
+  </si>
+  <si>
+    <t>1405/04/13</t>
+  </si>
+  <si>
+    <t>اصلاح دسترسی های واحد تعمیر و نگهداری بر اساس گروه</t>
+  </si>
+  <si>
+    <t>1405/01/25</t>
+  </si>
+  <si>
+    <t>فرم پاداش مصوب مدیریت</t>
+  </si>
+  <si>
+    <t>نوین شیمی</t>
+  </si>
+  <si>
+    <t>کاغذ آغشته</t>
+  </si>
+  <si>
+    <t>ایمنی و بهداشت</t>
+  </si>
+  <si>
+    <t>اصلاح گردش کار درخواست کالا و مرخصی/ماموریت</t>
+  </si>
+  <si>
+    <t>فرم پیمانکار و کارکرد پیمانکار</t>
+  </si>
+  <si>
+    <t>خرید چوب</t>
+  </si>
+  <si>
+    <t>1405/02/01</t>
+  </si>
+  <si>
+    <t>ساخت فرم کارکرد پیمانکاران جهت ثبت کارکرد ماشین آلات استیجاری</t>
+  </si>
+  <si>
+    <t>1405/02/06</t>
+  </si>
+  <si>
+    <t>فرم درخواست ماشین آلات</t>
+  </si>
+  <si>
+    <t>1405/03/09</t>
+  </si>
+  <si>
+    <t>ایجاد فرم درخواست ماشین آلات داخلی جهت ثبت نوبت</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -149,6 +410,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -197,7 +461,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -232,7 +496,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -441,7 +705,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.85546875" style="1" customWidth="1"/>
@@ -471,19 +735,19 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -494,38 +758,38 @@
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>17</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>110</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>11</v>
@@ -534,32 +798,32 @@
         <v>6</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>20</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>65</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>1</v>
+        <v>66</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>11</v>
@@ -568,46 +832,611 @@
         <v>6</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>27</v>
+      <c r="C34" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E31">
+    <sortState ref="A3:E30">
+      <sortCondition ref="B3"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>